<commit_message>
refactor: move bert_classifier module from notebooks to src directory
- Relocate bert_classifier.py to standard src structure for better project organization
- Remove duplicate file from notebooks directory to maintain single source of truth
- Update file paths to follow conventional Python project layout
</commit_message>
<xml_diff>
--- a/results/cobacek_compare_20datates.xlsx
+++ b/results/cobacek_compare_20datates.xlsx
@@ -10,6 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Predictions_Compare" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Metrics" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Category_Analysis" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -234,22 +235,37 @@
     </comment>
     <comment ref="U1" authorId="0" shapeId="0">
       <text>
+        <t>TRUE jika Hybrid SVM (gpt_5_4_mini) benar di category DAN priority sekaligus</t>
+      </text>
+    </comment>
+    <comment ref="V1" authorId="0" shapeId="0">
+      <text>
         <t>Prediksi kategori Hybrid SVM: SVM dikoreksi GenAI (gpt_4_1_mini) untuk baris mismatch</t>
       </text>
     </comment>
-    <comment ref="V1" authorId="0" shapeId="0">
+    <comment ref="W1" authorId="0" shapeId="0">
       <text>
         <t>Prediksi prioritas Hybrid SVM: SVM dikoreksi GenAI (gpt_4_1_mini) untuk baris mismatch</t>
       </text>
     </comment>
-    <comment ref="W1" authorId="0" shapeId="0">
+    <comment ref="X1" authorId="0" shapeId="0">
+      <text>
+        <t>TRUE jika Hybrid SVM (gpt_4_1_mini) benar di category DAN priority sekaligus</t>
+      </text>
+    </comment>
+    <comment ref="Y1" authorId="0" shapeId="0">
       <text>
         <t>Prediksi kategori Hybrid SVM: SVM dikoreksi GenAI (gpt_4o_mini) untuk baris mismatch</t>
       </text>
     </comment>
-    <comment ref="X1" authorId="0" shapeId="0">
+    <comment ref="Z1" authorId="0" shapeId="0">
       <text>
         <t>Prediksi prioritas Hybrid SVM: SVM dikoreksi GenAI (gpt_4o_mini) untuk baris mismatch</t>
+      </text>
+    </comment>
+    <comment ref="AA1" authorId="0" shapeId="0">
+      <text>
+        <t>TRUE jika Hybrid SVM (gpt_4o_mini) benar di category DAN priority sekaligus</t>
       </text>
     </comment>
   </commentList>
@@ -325,6 +341,66 @@
     <comment ref="B1" authorId="0" shapeId="0">
       <text>
         <t>Nilai dari parameter konfigurasi tersebut</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments/comment4.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>System</author>
+  </authors>
+  <commentList>
+    <comment ref="A1" authorId="0" shapeId="0">
+      <text>
+        <t>Nama kategori tiket helpdesk</t>
+      </text>
+    </comment>
+    <comment ref="B1" authorId="0" shapeId="0">
+      <text>
+        <t>Jumlah sampel (baris) untuk kategori ini dalam dataset</t>
+      </text>
+    </comment>
+    <comment ref="C1" authorId="0" shapeId="0">
+      <text>
+        <t>Akurasi prediksi kategori oleh SVM untuk kategori ini (benar / jumlah sampel)</t>
+      </text>
+    </comment>
+    <comment ref="D1" authorId="0" shapeId="0">
+      <text>
+        <t>Akurasi prediksi kategori oleh RF untuk kategori ini (benar / jumlah sampel)</t>
+      </text>
+    </comment>
+    <comment ref="E1" authorId="0" shapeId="0">
+      <text>
+        <t>Akurasi prediksi kategori oleh LR untuk kategori ini (benar / jumlah sampel)</t>
+      </text>
+    </comment>
+    <comment ref="F1" authorId="0" shapeId="0">
+      <text>
+        <t>Akurasi prediksi kategori oleh BERT untuk kategori ini (benar / jumlah sampel)</t>
+      </text>
+    </comment>
+    <comment ref="G1" authorId="0" shapeId="0">
+      <text>
+        <t>Akurasi prediksi kategori oleh Hybrid (gpt-5.4-mini) untuk kategori ini (benar / jumlah sampel)</t>
+      </text>
+    </comment>
+    <comment ref="H1" authorId="0" shapeId="0">
+      <text>
+        <t>Akurasi prediksi kategori oleh Hybrid (gpt-4.1-mini) untuk kategori ini (benar / jumlah sampel)</t>
+      </text>
+    </comment>
+    <comment ref="I1" authorId="0" shapeId="0">
+      <text>
+        <t>Akurasi prediksi kategori oleh Hybrid (gpt-4o-mini) untuk kategori ini (benar / jumlah sampel)</t>
+      </text>
+    </comment>
+    <comment ref="J1" authorId="0" shapeId="0">
+      <text>
+        <t>Model dengan akurasi tertinggi untuk kategori ini (bisa N/A jika semua model gagal)</t>
       </text>
     </comment>
   </commentList>
@@ -620,7 +696,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X21"/>
+  <dimension ref="A1:AA21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -726,22 +802,37 @@
       </c>
       <c r="U1" t="inlineStr">
         <is>
+          <t>hybrid_svm_match_gpt_5_4_mini</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
           <t>hybrid_svm_category_gpt_4_1_mini</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>hybrid_svm_priority_gpt_4_1_mini</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="X1" t="inlineStr">
+        <is>
+          <t>hybrid_svm_match_gpt_4_1_mini</t>
+        </is>
+      </c>
+      <c r="Y1" t="inlineStr">
         <is>
           <t>hybrid_svm_category_gpt_4o_mini</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>hybrid_svm_priority_gpt_4o_mini</t>
+        </is>
+      </c>
+      <c r="AA1" t="inlineStr">
+        <is>
+          <t>hybrid_svm_match_gpt_4o_mini</t>
         </is>
       </c>
     </row>
@@ -817,7 +908,7 @@
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>Network</t>
+          <t>Product</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
@@ -838,25 +929,34 @@
           <t>high</t>
         </is>
       </c>
-      <c r="U2" t="inlineStr">
+      <c r="U2" t="b">
+        <v>0</v>
+      </c>
+      <c r="V2" t="inlineStr">
         <is>
           <t>Outage</t>
         </is>
       </c>
-      <c r="V2" t="inlineStr">
+      <c r="W2" t="inlineStr">
         <is>
           <t>high</t>
         </is>
       </c>
-      <c r="W2" t="inlineStr">
+      <c r="X2" t="b">
+        <v>0</v>
+      </c>
+      <c r="Y2" t="inlineStr">
         <is>
           <t>Outage</t>
         </is>
       </c>
-      <c r="X2" t="inlineStr">
+      <c r="Z2" t="inlineStr">
         <is>
           <t>high</t>
         </is>
+      </c>
+      <c r="AA2" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -931,7 +1031,7 @@
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>Product</t>
+          <t>Inquiry</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
@@ -940,7 +1040,7 @@
         </is>
       </c>
       <c r="R3" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S3" t="inlineStr">
         <is>
@@ -952,25 +1052,34 @@
           <t>medium</t>
         </is>
       </c>
-      <c r="U3" t="inlineStr">
-        <is>
-          <t>Product</t>
-        </is>
+      <c r="U3" t="b">
+        <v>1</v>
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>Product</t>
         </is>
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>Product</t>
-        </is>
-      </c>
-      <c r="X3" t="inlineStr">
-        <is>
-          <t>medium</t>
-        </is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="X3" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y3" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="Z3" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="AA3" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="4">
@@ -1045,7 +1154,7 @@
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>Marketing</t>
+          <t>Feature</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
@@ -1066,25 +1175,34 @@
           <t>low</t>
         </is>
       </c>
-      <c r="U4" t="inlineStr">
+      <c r="U4" t="b">
+        <v>1</v>
+      </c>
+      <c r="V4" t="inlineStr">
         <is>
           <t>Billing</t>
         </is>
       </c>
-      <c r="V4" t="inlineStr">
+      <c r="W4" t="inlineStr">
         <is>
           <t>low</t>
         </is>
       </c>
-      <c r="W4" t="inlineStr">
+      <c r="X4" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y4" t="inlineStr">
         <is>
           <t>Billing</t>
         </is>
       </c>
-      <c r="X4" t="inlineStr">
-        <is>
-          <t>medium</t>
-        </is>
+      <c r="Z4" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="AA4" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -1159,12 +1277,12 @@
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>Disruption</t>
+          <t>Product</t>
         </is>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="R5" t="b">
@@ -1180,25 +1298,34 @@
           <t>medium</t>
         </is>
       </c>
-      <c r="U5" t="inlineStr">
-        <is>
-          <t>Product</t>
-        </is>
+      <c r="U5" t="b">
+        <v>1</v>
       </c>
       <c r="V5" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>Product</t>
         </is>
       </c>
       <c r="W5" t="inlineStr">
         <is>
-          <t>Product</t>
-        </is>
-      </c>
-      <c r="X5" t="inlineStr">
-        <is>
-          <t>medium</t>
-        </is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="X5" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y5" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="Z5" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="AA5" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="6">
@@ -1273,7 +1400,7 @@
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>Marketing</t>
+          <t>Feature</t>
         </is>
       </c>
       <c r="Q6" t="inlineStr">
@@ -1294,25 +1421,34 @@
           <t>low</t>
         </is>
       </c>
-      <c r="U6" t="inlineStr">
+      <c r="U6" t="b">
+        <v>0</v>
+      </c>
+      <c r="V6" t="inlineStr">
         <is>
           <t>Inquiry</t>
         </is>
       </c>
-      <c r="V6" t="inlineStr">
+      <c r="W6" t="inlineStr">
         <is>
           <t>low</t>
         </is>
       </c>
-      <c r="W6" t="inlineStr">
+      <c r="X6" t="b">
+        <v>0</v>
+      </c>
+      <c r="Y6" t="inlineStr">
         <is>
           <t>Inquiry</t>
         </is>
       </c>
-      <c r="X6" t="inlineStr">
-        <is>
-          <t>low</t>
-        </is>
+      <c r="Z6" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="AA6" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="7">
@@ -1387,46 +1523,55 @@
       </c>
       <c r="P7" t="inlineStr">
         <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="R7" t="b">
+        <v>0</v>
+      </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>Outage</t>
+        </is>
+      </c>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="U7" t="b">
+        <v>1</v>
+      </c>
+      <c r="V7" t="inlineStr">
+        <is>
+          <t>Outage</t>
+        </is>
+      </c>
+      <c r="W7" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="X7" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y7" t="inlineStr">
+        <is>
           <t>Disruption</t>
         </is>
       </c>
-      <c r="Q7" t="inlineStr">
-        <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="R7" t="b">
-        <v>0</v>
-      </c>
-      <c r="S7" t="inlineStr">
-        <is>
-          <t>Network</t>
-        </is>
-      </c>
-      <c r="T7" t="inlineStr">
+      <c r="Z7" t="inlineStr">
         <is>
           <t>high</t>
         </is>
       </c>
-      <c r="U7" t="inlineStr">
-        <is>
-          <t>Outage</t>
-        </is>
-      </c>
-      <c r="V7" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="W7" t="inlineStr">
-        <is>
-          <t>Disruption</t>
-        </is>
-      </c>
-      <c r="X7" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
+      <c r="AA7" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="8">
@@ -1501,7 +1646,7 @@
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>Network</t>
+          <t>Feature</t>
         </is>
       </c>
       <c r="Q8" t="inlineStr">
@@ -1510,7 +1655,7 @@
         </is>
       </c>
       <c r="R8" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S8" t="inlineStr">
         <is>
@@ -1522,25 +1667,34 @@
           <t>medium</t>
         </is>
       </c>
-      <c r="U8" t="inlineStr">
+      <c r="U8" t="b">
+        <v>0</v>
+      </c>
+      <c r="V8" t="inlineStr">
         <is>
           <t>Bug</t>
         </is>
       </c>
-      <c r="V8" t="inlineStr">
-        <is>
-          <t>medium</t>
-        </is>
-      </c>
       <c r="W8" t="inlineStr">
         <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="X8" t="b">
+        <v>0</v>
+      </c>
+      <c r="Y8" t="inlineStr">
+        <is>
           <t>Bug</t>
         </is>
       </c>
-      <c r="X8" t="inlineStr">
+      <c r="Z8" t="inlineStr">
         <is>
           <t>high</t>
         </is>
+      </c>
+      <c r="AA8" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="9">
@@ -1615,7 +1769,7 @@
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>Disruption</t>
+          <t>Product</t>
         </is>
       </c>
       <c r="Q9" t="inlineStr">
@@ -1636,25 +1790,34 @@
           <t>medium</t>
         </is>
       </c>
-      <c r="U9" t="inlineStr">
+      <c r="U9" t="b">
+        <v>1</v>
+      </c>
+      <c r="V9" t="inlineStr">
         <is>
           <t>Network</t>
         </is>
       </c>
-      <c r="V9" t="inlineStr">
-        <is>
-          <t>medium</t>
-        </is>
-      </c>
       <c r="W9" t="inlineStr">
         <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="X9" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y9" t="inlineStr">
+        <is>
           <t>Network</t>
         </is>
       </c>
-      <c r="X9" t="inlineStr">
-        <is>
-          <t>medium</t>
-        </is>
+      <c r="Z9" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="AA9" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="10">
@@ -1729,7 +1892,7 @@
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>Product</t>
+          <t>Inquiry</t>
         </is>
       </c>
       <c r="Q10" t="inlineStr">
@@ -1750,25 +1913,34 @@
           <t>high</t>
         </is>
       </c>
-      <c r="U10" t="inlineStr">
+      <c r="U10" t="b">
+        <v>0</v>
+      </c>
+      <c r="V10" t="inlineStr">
         <is>
           <t>Disruption</t>
         </is>
       </c>
-      <c r="V10" t="inlineStr">
+      <c r="W10" t="inlineStr">
         <is>
           <t>high</t>
         </is>
       </c>
-      <c r="W10" t="inlineStr">
+      <c r="X10" t="b">
+        <v>0</v>
+      </c>
+      <c r="Y10" t="inlineStr">
         <is>
           <t>Disruption</t>
         </is>
       </c>
-      <c r="X10" t="inlineStr">
+      <c r="Z10" t="inlineStr">
         <is>
           <t>high</t>
         </is>
+      </c>
+      <c r="AA10" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="11">
@@ -1843,7 +2015,7 @@
       </c>
       <c r="P11" t="inlineStr">
         <is>
-          <t>Marketing</t>
+          <t>Billing</t>
         </is>
       </c>
       <c r="Q11" t="inlineStr">
@@ -1864,25 +2036,34 @@
           <t>low</t>
         </is>
       </c>
-      <c r="U11" t="inlineStr">
+      <c r="U11" t="b">
+        <v>0</v>
+      </c>
+      <c r="V11" t="inlineStr">
         <is>
           <t>Inquiry</t>
         </is>
       </c>
-      <c r="V11" t="inlineStr">
+      <c r="W11" t="inlineStr">
         <is>
           <t>low</t>
         </is>
       </c>
-      <c r="W11" t="inlineStr">
+      <c r="X11" t="b">
+        <v>0</v>
+      </c>
+      <c r="Y11" t="inlineStr">
         <is>
           <t>Inquiry</t>
         </is>
       </c>
-      <c r="X11" t="inlineStr">
-        <is>
-          <t>medium</t>
-        </is>
+      <c r="Z11" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="AA11" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="12">
@@ -1957,7 +2138,7 @@
       </c>
       <c r="P12" t="inlineStr">
         <is>
-          <t>Product</t>
+          <t>Billing</t>
         </is>
       </c>
       <c r="Q12" t="inlineStr">
@@ -1978,25 +2159,34 @@
           <t>medium</t>
         </is>
       </c>
-      <c r="U12" t="inlineStr">
+      <c r="U12" t="b">
+        <v>1</v>
+      </c>
+      <c r="V12" t="inlineStr">
         <is>
           <t>Bug</t>
         </is>
       </c>
-      <c r="V12" t="inlineStr">
-        <is>
-          <t>medium</t>
-        </is>
-      </c>
       <c r="W12" t="inlineStr">
         <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="X12" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y12" t="inlineStr">
+        <is>
           <t>Bug</t>
         </is>
       </c>
-      <c r="X12" t="inlineStr">
-        <is>
-          <t>medium</t>
-        </is>
+      <c r="Z12" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="AA12" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="13">
@@ -2071,7 +2261,7 @@
       </c>
       <c r="P13" t="inlineStr">
         <is>
-          <t>Disruption</t>
+          <t>Product</t>
         </is>
       </c>
       <c r="Q13" t="inlineStr">
@@ -2092,25 +2282,34 @@
           <t>low</t>
         </is>
       </c>
-      <c r="U13" t="inlineStr">
+      <c r="U13" t="b">
+        <v>0</v>
+      </c>
+      <c r="V13" t="inlineStr">
         <is>
           <t>Inquiry</t>
         </is>
       </c>
-      <c r="V13" t="inlineStr">
+      <c r="W13" t="inlineStr">
         <is>
           <t>low</t>
         </is>
       </c>
-      <c r="W13" t="inlineStr">
+      <c r="X13" t="b">
+        <v>0</v>
+      </c>
+      <c r="Y13" t="inlineStr">
         <is>
           <t>Inquiry</t>
         </is>
       </c>
-      <c r="X13" t="inlineStr">
-        <is>
-          <t>medium</t>
-        </is>
+      <c r="Z13" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="AA13" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="14">
@@ -2185,7 +2384,7 @@
       </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t>Product</t>
+          <t>Inquiry</t>
         </is>
       </c>
       <c r="Q14" t="inlineStr">
@@ -2206,25 +2405,34 @@
           <t>low</t>
         </is>
       </c>
-      <c r="U14" t="inlineStr">
+      <c r="U14" t="b">
+        <v>0</v>
+      </c>
+      <c r="V14" t="inlineStr">
         <is>
           <t>Marketing</t>
         </is>
       </c>
-      <c r="V14" t="inlineStr">
-        <is>
-          <t>medium</t>
-        </is>
-      </c>
       <c r="W14" t="inlineStr">
         <is>
-          <t>Marketing</t>
-        </is>
-      </c>
-      <c r="X14" t="inlineStr">
-        <is>
-          <t>medium</t>
-        </is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="X14" t="b">
+        <v>0</v>
+      </c>
+      <c r="Y14" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="Z14" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="AA14" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="15">
@@ -2299,7 +2507,7 @@
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>Product</t>
+          <t>Inquiry</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
@@ -2320,25 +2528,34 @@
           <t>low</t>
         </is>
       </c>
-      <c r="U15" t="inlineStr">
+      <c r="U15" t="b">
+        <v>0</v>
+      </c>
+      <c r="V15" t="inlineStr">
         <is>
           <t>Marketing</t>
         </is>
       </c>
-      <c r="V15" t="inlineStr">
+      <c r="W15" t="inlineStr">
         <is>
           <t>low</t>
         </is>
       </c>
-      <c r="W15" t="inlineStr">
+      <c r="X15" t="b">
+        <v>0</v>
+      </c>
+      <c r="Y15" t="inlineStr">
         <is>
           <t>Marketing</t>
         </is>
       </c>
-      <c r="X15" t="inlineStr">
-        <is>
-          <t>medium</t>
-        </is>
+      <c r="Z15" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="AA15" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="16">
@@ -2413,7 +2630,7 @@
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>Product</t>
+          <t>Billing</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
@@ -2431,28 +2648,37 @@
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="U16" t="inlineStr">
+          <t>low</t>
+        </is>
+      </c>
+      <c r="U16" t="b">
+        <v>0</v>
+      </c>
+      <c r="V16" t="inlineStr">
         <is>
           <t>Disruption</t>
         </is>
       </c>
-      <c r="V16" t="inlineStr">
-        <is>
-          <t>medium</t>
-        </is>
-      </c>
       <c r="W16" t="inlineStr">
         <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="X16" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y16" t="inlineStr">
+        <is>
           <t>Disruption</t>
         </is>
       </c>
-      <c r="X16" t="inlineStr">
+      <c r="Z16" t="inlineStr">
         <is>
           <t>high</t>
         </is>
+      </c>
+      <c r="AA16" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="17">
@@ -2527,7 +2753,7 @@
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>Product</t>
+          <t>Inquiry</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
@@ -2548,25 +2774,34 @@
           <t>low</t>
         </is>
       </c>
-      <c r="U17" t="inlineStr">
+      <c r="U17" t="b">
+        <v>0</v>
+      </c>
+      <c r="V17" t="inlineStr">
         <is>
           <t>Feature</t>
         </is>
       </c>
-      <c r="V17" t="inlineStr">
-        <is>
-          <t>medium</t>
-        </is>
-      </c>
       <c r="W17" t="inlineStr">
         <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="X17" t="b">
+        <v>0</v>
+      </c>
+      <c r="Y17" t="inlineStr">
+        <is>
           <t>Feature</t>
         </is>
       </c>
-      <c r="X17" t="inlineStr">
-        <is>
-          <t>medium</t>
-        </is>
+      <c r="Z17" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="AA17" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="18">
@@ -2641,16 +2876,16 @@
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>Account</t>
+          <t>Product</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="R18" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S18" t="inlineStr">
         <is>
@@ -2662,25 +2897,34 @@
           <t>low</t>
         </is>
       </c>
-      <c r="U18" t="inlineStr">
+      <c r="U18" t="b">
+        <v>0</v>
+      </c>
+      <c r="V18" t="inlineStr">
         <is>
           <t>Inquiry</t>
         </is>
       </c>
-      <c r="V18" t="inlineStr">
-        <is>
-          <t>medium</t>
-        </is>
-      </c>
       <c r="W18" t="inlineStr">
         <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="X18" t="b">
+        <v>0</v>
+      </c>
+      <c r="Y18" t="inlineStr">
+        <is>
           <t>Inquiry</t>
         </is>
       </c>
-      <c r="X18" t="inlineStr">
-        <is>
-          <t>medium</t>
-        </is>
+      <c r="Z18" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="AA18" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="19">
@@ -2776,25 +3020,34 @@
           <t>medium</t>
         </is>
       </c>
-      <c r="U19" t="inlineStr">
+      <c r="U19" t="b">
+        <v>0</v>
+      </c>
+      <c r="V19" t="inlineStr">
+        <is>
+          <t>Disruption</t>
+        </is>
+      </c>
+      <c r="W19" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="X19" t="b">
+        <v>0</v>
+      </c>
+      <c r="Y19" t="inlineStr">
         <is>
           <t>Bug</t>
         </is>
       </c>
-      <c r="V19" t="inlineStr">
+      <c r="Z19" t="inlineStr">
         <is>
           <t>high</t>
         </is>
       </c>
-      <c r="W19" t="inlineStr">
-        <is>
-          <t>Bug</t>
-        </is>
-      </c>
-      <c r="X19" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
+      <c r="AA19" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="20">
@@ -2869,12 +3122,12 @@
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>Account</t>
+          <t>Product</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="R20" t="b">
@@ -2890,25 +3143,34 @@
           <t>low</t>
         </is>
       </c>
-      <c r="U20" t="inlineStr">
+      <c r="U20" t="b">
+        <v>0</v>
+      </c>
+      <c r="V20" t="inlineStr">
         <is>
           <t>Billing</t>
         </is>
       </c>
-      <c r="V20" t="inlineStr">
-        <is>
-          <t>medium</t>
-        </is>
-      </c>
       <c r="W20" t="inlineStr">
         <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="X20" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y20" t="inlineStr">
+        <is>
           <t>Billing</t>
         </is>
       </c>
-      <c r="X20" t="inlineStr">
-        <is>
-          <t>medium</t>
-        </is>
+      <c r="Z20" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="AA20" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="21">
@@ -2983,7 +3245,7 @@
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t>Disruption</t>
+          <t>Inquiry</t>
         </is>
       </c>
       <c r="Q21" t="inlineStr">
@@ -3004,25 +3266,34 @@
           <t>medium</t>
         </is>
       </c>
-      <c r="U21" t="inlineStr">
+      <c r="U21" t="b">
+        <v>1</v>
+      </c>
+      <c r="V21" t="inlineStr">
         <is>
           <t>Network</t>
         </is>
       </c>
-      <c r="V21" t="inlineStr">
-        <is>
-          <t>medium</t>
-        </is>
-      </c>
       <c r="W21" t="inlineStr">
         <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="X21" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y21" t="inlineStr">
+        <is>
           <t>Network</t>
         </is>
       </c>
-      <c r="X21" t="inlineStr">
-        <is>
-          <t>medium</t>
-        </is>
+      <c r="Z21" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="AA21" t="b">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -3094,7 +3365,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.09</v>
+        <v>0.23</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -3127,7 +3398,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.09</v>
+        <v>0.23</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -3160,7 +3431,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>3.93</v>
+        <v>10.1</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -3193,7 +3464,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>3.93</v>
+        <v>10.1</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -3226,7 +3497,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.24</v>
+        <v>0.64</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -3259,7 +3530,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.24</v>
+        <v>0.64</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -3292,7 +3563,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>53.74</v>
+        <v>63.11</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -3303,16 +3574,16 @@
         <v>0.15</v>
       </c>
       <c r="E8" t="n">
-        <v>0.075</v>
+        <v>0.05833333333333333</v>
       </c>
       <c r="F8" t="n">
-        <v>0.07333333333333333</v>
+        <v>0.09</v>
       </c>
       <c r="G8" t="n">
         <v>0.07076923076923078</v>
       </c>
       <c r="H8" t="n">
-        <v>0.1369230769230769</v>
+        <v>0.1169230769230769</v>
       </c>
       <c r="I8" t="n">
         <v>20</v>
@@ -3325,7 +3596,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>53.74</v>
+        <v>63.11</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -3336,16 +3607,16 @@
         <v>0.55</v>
       </c>
       <c r="E9" t="n">
-        <v>0.1833333333333333</v>
+        <v>0.3541666666666667</v>
       </c>
       <c r="F9" t="n">
+        <v>0.3560606060606061</v>
+      </c>
+      <c r="G9" t="n">
         <v>0.3333333333333333</v>
       </c>
-      <c r="G9" t="n">
-        <v>0.2365591397849462</v>
-      </c>
       <c r="H9" t="n">
-        <v>0.3903225806451613</v>
+        <v>0.5</v>
       </c>
       <c r="I9" t="n">
         <v>20</v>
@@ -3358,7 +3629,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>23.27</v>
+        <v>19.28</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -3366,19 +3637,19 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>0.4</v>
+        <v>0.45</v>
       </c>
       <c r="E10" t="n">
-        <v>0.3142857142857143</v>
+        <v>0.3976190476190476</v>
       </c>
       <c r="F10" t="n">
-        <v>0.3566666666666666</v>
+        <v>0.4566666666666667</v>
       </c>
       <c r="G10" t="n">
-        <v>0.2888095238095237</v>
+        <v>0.3688095238095238</v>
       </c>
       <c r="H10" t="n">
-        <v>0.3953571428571429</v>
+        <v>0.4486904761904763</v>
       </c>
       <c r="I10" t="n">
         <v>20</v>
@@ -3391,7 +3662,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>23.27</v>
+        <v>19.28</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -3399,19 +3670,19 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>0.5</v>
+        <v>0.45</v>
       </c>
       <c r="E11" t="n">
-        <v>0.5509259259259259</v>
+        <v>0.5412698412698412</v>
       </c>
       <c r="F11" t="n">
-        <v>0.6287878787878788</v>
+        <v>0.5984848484848485</v>
       </c>
       <c r="G11" t="n">
-        <v>0.4334928229665072</v>
+        <v>0.404040404040404</v>
       </c>
       <c r="H11" t="n">
-        <v>0.5607177033492823</v>
+        <v>0.5212121212121212</v>
       </c>
       <c r="I11" t="n">
         <v>20</v>
@@ -3424,7 +3695,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>23.6</v>
+        <v>22.36</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -3441,10 +3712,10 @@
         <v>0.6566666666666666</v>
       </c>
       <c r="G12" t="n">
-        <v>0.5171428571428571</v>
+        <v>0.5104761904761904</v>
       </c>
       <c r="H12" t="n">
-        <v>0.5228571428571429</v>
+        <v>0.5245238095238095</v>
       </c>
       <c r="I12" t="n">
         <v>20</v>
@@ -3457,7 +3728,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>23.6</v>
+        <v>22.36</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -3468,16 +3739,16 @@
         <v>0.6</v>
       </c>
       <c r="E13" t="n">
-        <v>0.5590909090909091</v>
+        <v>0.5939153439153438</v>
       </c>
       <c r="F13" t="n">
         <v>0.7007575757575758</v>
       </c>
       <c r="G13" t="n">
-        <v>0.5202020202020202</v>
+        <v>0.5166666666666667</v>
       </c>
       <c r="H13" t="n">
-        <v>0.6166666666666666</v>
+        <v>0.6525000000000001</v>
       </c>
       <c r="I13" t="n">
         <v>20</v>
@@ -3490,7 +3761,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>23.69</v>
+        <v>25.58</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -3498,19 +3769,19 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>0.5</v>
+        <v>0.55</v>
       </c>
       <c r="E14" t="n">
-        <v>0.4416666666666666</v>
+        <v>0.5416666666666666</v>
       </c>
       <c r="F14" t="n">
-        <v>0.5566666666666666</v>
+        <v>0.6066666666666667</v>
       </c>
       <c r="G14" t="n">
-        <v>0.4338095238095238</v>
+        <v>0.5171428571428571</v>
       </c>
       <c r="H14" t="n">
-        <v>0.4811904761904762</v>
+        <v>0.5478571428571429</v>
       </c>
       <c r="I14" t="n">
         <v>20</v>
@@ -3523,7 +3794,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>23.69</v>
+        <v>25.58</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -3534,16 +3805,16 @@
         <v>0.55</v>
       </c>
       <c r="E15" t="n">
-        <v>0.3717948717948718</v>
+        <v>0.3571428571428572</v>
       </c>
       <c r="F15" t="n">
         <v>0.3674242424242424</v>
       </c>
       <c r="G15" t="n">
-        <v>0.3650793650793651</v>
+        <v>0.3561904761904762</v>
       </c>
       <c r="H15" t="n">
-        <v>0.5380952380952381</v>
+        <v>0.5234285714285714</v>
       </c>
       <c r="I15" t="n">
         <v>20</v>
@@ -3634,4 +3905,431 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>category</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>acc_SVM</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>acc_RF</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>acc_LR</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>acc_BERT</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>acc_Hybrid (gpt-5.4-mini)</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>acc_Hybrid (gpt-4.1-mini)</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>acc_Hybrid (gpt-4o-mini)</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>best_model</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>5</v>
+      </c>
+      <c r="C2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>SVM</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Network</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>3</v>
+      </c>
+      <c r="C3" t="n">
+        <v>0.6667</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0.3333</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0.6667</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0.6667</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0.6667</v>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>SVM</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Billing</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>2</v>
+      </c>
+      <c r="C4" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I4" t="n">
+        <v>1</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Hybrid (gpt-5.4-mini)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Account</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>2</v>
+      </c>
+      <c r="C5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Bug</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>2</v>
+      </c>
+      <c r="C6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="I6" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Hybrid (gpt-5.4-mini)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>2</v>
+      </c>
+      <c r="C7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>BERT</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Inquiry</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>1</v>
+      </c>
+      <c r="C8" t="n">
+        <v>0</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" t="n">
+        <v>1</v>
+      </c>
+      <c r="H8" t="n">
+        <v>1</v>
+      </c>
+      <c r="I8" t="n">
+        <v>1</v>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Hybrid (gpt-5.4-mini)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Disruption</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>1</v>
+      </c>
+      <c r="C9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" t="n">
+        <v>1</v>
+      </c>
+      <c r="I9" t="n">
+        <v>1</v>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Hybrid (gpt-4.1-mini)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Marketing</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>1</v>
+      </c>
+      <c r="C10" t="n">
+        <v>0</v>
+      </c>
+      <c r="D10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" t="n">
+        <v>1</v>
+      </c>
+      <c r="I10" t="n">
+        <v>1</v>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Hybrid (gpt-4.1-mini)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Outage</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>1</v>
+      </c>
+      <c r="C11" t="n">
+        <v>0</v>
+      </c>
+      <c r="D11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" t="n">
+        <v>1</v>
+      </c>
+      <c r="H11" t="n">
+        <v>1</v>
+      </c>
+      <c r="I11" t="n">
+        <v>0</v>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Hybrid (gpt-5.4-mini)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
+</worksheet>
 </file>
</xml_diff>